<commit_message>
update call llm with multiple provider, langraph for tool calling, chat
</commit_message>
<xml_diff>
--- a/docs/ke-hoach-backend-8-tuan.xlsx
+++ b/docs/ke-hoach-backend-8-tuan.xlsx
@@ -915,9 +915,9 @@
       <c r="I2" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="J2" s="9" t="inlineStr">
-        <is>
-          <t>Chưa bắt đầu</t>
+      <c r="J2" s="16" t="inlineStr">
+        <is>
+          <t>Xong</t>
         </is>
       </c>
     </row>

</xml_diff>